<commit_message>
added measurment versus model results
</commit_message>
<xml_diff>
--- a/modelling/wsf grondwaterstroming/Properties_calculator.xlsx
+++ b/modelling/wsf grondwaterstroming/Properties_calculator.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Gitclones\FusionFiber\modelling\wsf grondwaterstroming\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2588B3D0-34A3-45A9-A87C-5AA277EEC78B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C73F58B-E895-430C-9518-F46736A27C13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{3632657A-28F7-4C1C-ABB4-32E130E65C30}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="71">
   <si>
     <t>n</t>
   </si>
@@ -213,6 +213,42 @@
   </si>
   <si>
     <t>Rtotal</t>
+  </si>
+  <si>
+    <t>gw300</t>
+  </si>
+  <si>
+    <t>Expected conductivty</t>
+  </si>
+  <si>
+    <t>gw301</t>
+  </si>
+  <si>
+    <t>gw302</t>
+  </si>
+  <si>
+    <t>gw303</t>
+  </si>
+  <si>
+    <t>gw304</t>
+  </si>
+  <si>
+    <t>gw305</t>
+  </si>
+  <si>
+    <t>gw306</t>
+  </si>
+  <si>
+    <t>gw307</t>
+  </si>
+  <si>
+    <t>gw308</t>
+  </si>
+  <si>
+    <t>gw309</t>
+  </si>
+  <si>
+    <t>gw310</t>
   </si>
 </sst>
 </file>
@@ -275,23 +311,27 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
+      <sz val="8"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor theme="4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -299,11 +339,57 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color theme="4"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color theme="4"/>
+      </right>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -333,17 +419,59 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="15">
+  <dxfs count="16">
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
     <dxf>
       <font>
         <b/>
@@ -356,16 +484,13 @@
         <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="11"/>
-        <color theme="4"/>
+        <color auto="1"/>
         <name val="Aptos Narrow"/>
         <family val="2"/>
         <scheme val="minor"/>
       </font>
-      <numFmt numFmtId="2" formatCode="0.00"/>
+      <numFmt numFmtId="164" formatCode="0.000"/>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
       <font>
@@ -462,6 +587,26 @@
         <family val="2"/>
         <scheme val="minor"/>
       </font>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="4"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="2" formatCode="0.00"/>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -607,13 +752,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>16</xdr:col>
+      <xdr:col>17</xdr:col>
       <xdr:colOff>164124</xdr:colOff>
       <xdr:row>17</xdr:row>
       <xdr:rowOff>169984</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>19</xdr:col>
+      <xdr:col>20</xdr:col>
       <xdr:colOff>572059</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>8186</xdr:rowOff>
@@ -659,14 +804,14 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>15</xdr:col>
+      <xdr:col>16</xdr:col>
       <xdr:colOff>785447</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>169982</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>20</xdr:col>
-      <xdr:colOff>781722</xdr:colOff>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>575982</xdr:colOff>
       <xdr:row>27</xdr:row>
       <xdr:rowOff>167554</xdr:rowOff>
     </xdr:to>
@@ -710,18 +855,18 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{61B2F13E-E38A-4556-AD9E-4A31FC65E5B2}" name="Table134" displayName="Table134" ref="A17:O26" totalsRowShown="0" headerRowDxfId="14">
-  <autoFilter ref="A17:O26" xr:uid="{61B2F13E-E38A-4556-AD9E-4A31FC65E5B2}"/>
-  <tableColumns count="15">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{61B2F13E-E38A-4556-AD9E-4A31FC65E5B2}" name="Table134" displayName="Table134" ref="A17:P27" totalsRowShown="0" headerRowDxfId="15">
+  <autoFilter ref="A17:P27" xr:uid="{61B2F13E-E38A-4556-AD9E-4A31FC65E5B2}"/>
+  <tableColumns count="16">
     <tableColumn id="1" xr3:uid="{D88FD9F6-4197-4562-AEB5-6E64BB7B60DF}" name="test_id"/>
-    <tableColumn id="2" xr3:uid="{60857CD5-5FC9-4195-B59E-DCF7E4200979}" name="voltage" dataDxfId="13"/>
-    <tableColumn id="3" xr3:uid="{DC49E5D0-E51E-4B30-8721-2B94794996C4}" name="R' " dataDxfId="12"/>
-    <tableColumn id="4" xr3:uid="{D3B11A5D-6B20-4BAD-9548-D20A742D41CD}" name="L_heat" dataDxfId="11"/>
-    <tableColumn id="5" xr3:uid="{4584E915-A1FB-40E2-8D9A-AF0AA3924EB8}" name="Rtotal" dataDxfId="10"/>
-    <tableColumn id="6" xr3:uid="{824832D0-1465-46BF-B1DB-BC3BB2B60BB1}" name="Q" dataDxfId="9">
+    <tableColumn id="2" xr3:uid="{60857CD5-5FC9-4195-B59E-DCF7E4200979}" name="voltage" dataDxfId="14"/>
+    <tableColumn id="3" xr3:uid="{DC49E5D0-E51E-4B30-8721-2B94794996C4}" name="R' " dataDxfId="13"/>
+    <tableColumn id="4" xr3:uid="{D3B11A5D-6B20-4BAD-9548-D20A742D41CD}" name="L_heat" dataDxfId="12"/>
+    <tableColumn id="5" xr3:uid="{4584E915-A1FB-40E2-8D9A-AF0AA3924EB8}" name="Rtotal" dataDxfId="11"/>
+    <tableColumn id="6" xr3:uid="{824832D0-1465-46BF-B1DB-BC3BB2B60BB1}" name="Q" dataDxfId="10">
       <calculatedColumnFormula>#REF!/D18</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="15" xr3:uid="{EA6FF7B3-D4B1-4528-B1DE-055780E0D12E}" name="ncores" dataDxfId="0"/>
+    <tableColumn id="15" xr3:uid="{EA6FF7B3-D4B1-4528-B1DE-055780E0D12E}" name="ncores" dataDxfId="9"/>
     <tableColumn id="13" xr3:uid="{948E3691-0FA0-4A22-9288-16019CC9AC13}" name="Qtotal" dataDxfId="8"/>
     <tableColumn id="7" xr3:uid="{0EDD676B-B419-4ABD-9D3B-FA77118332A8}" name="4pi" dataDxfId="7">
       <calculatedColumnFormula>4*PI()</calculatedColumnFormula>
@@ -735,7 +880,8 @@
     <tableColumn id="12" xr3:uid="{592CBC98-0598-4037-9EBB-0C85EDD981BD}" name="themal conductivity" dataDxfId="2">
       <calculatedColumnFormula>(F18/(I18*J18))*M18</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="14" xr3:uid="{5268CFBE-FCA9-49F7-84B9-D28633D99E4F}" name="Relative error" dataDxfId="1">
+    <tableColumn id="16" xr3:uid="{B3214748-DDC5-499A-9049-D295CF923A61}" name="Expected conductivty" dataDxfId="1"/>
+    <tableColumn id="14" xr3:uid="{5268CFBE-FCA9-49F7-84B9-D28633D99E4F}" name="Relative error" dataDxfId="0">
       <calculatedColumnFormula>100*((Table134[[#This Row],[themal conductivity]]/1.6)-1)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1060,7 +1206,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EE086DA3-B7D9-4EBD-B1A4-5E6F632602CC}">
-  <dimension ref="A1:P26"/>
+  <dimension ref="A1:Q42"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="11" max="11" width="9.77734375" customWidth="1"/>
@@ -1241,7 +1387,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="17" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
         <v>42</v>
       </c>
@@ -1284,11 +1430,14 @@
       <c r="N17" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="O17" s="2" t="s">
+      <c r="O17" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="P17" s="2" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="18" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:17" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
         <v>3</v>
       </c>
@@ -1331,12 +1480,15 @@
       <c r="N18" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="O18" t="s">
+      <c r="O18" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="P18" t="s">
         <v>55</v>
       </c>
-      <c r="P18"/>
-    </row>
-    <row r="19" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q18"/>
+    </row>
+    <row r="19" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>29</v>
       </c>
@@ -1369,7 +1521,7 @@
         <v>12.566370614359172</v>
       </c>
       <c r="J19" s="14">
-        <v>1.81</v>
+        <v>4.7300000000000004</v>
       </c>
       <c r="K19" s="3">
         <v>600</v>
@@ -1383,14 +1535,17 @@
       </c>
       <c r="N19" s="11">
         <f>(H19/(I19*J19))*M19</f>
-        <v>4.2034305037403428</v>
-      </c>
-      <c r="O19" s="12">
+        <v>1.6085008904376361</v>
+      </c>
+      <c r="O19" s="11">
+        <v>1.6</v>
+      </c>
+      <c r="P19" s="12">
         <f>100*((Table134[[#This Row],[themal conductivity]]/1.6)-1)</f>
-        <v>162.71440648377143</v>
-      </c>
-    </row>
-    <row r="20" spans="1:16" x14ac:dyDescent="0.3">
+        <v>0.53130565235224303</v>
+      </c>
+    </row>
+    <row r="20" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>30</v>
       </c>
@@ -1423,7 +1578,7 @@
         <v>12.566370614359172</v>
       </c>
       <c r="J20" s="14">
-        <v>1.37</v>
+        <v>3.58</v>
       </c>
       <c r="K20" s="3">
         <v>600</v>
@@ -1437,14 +1592,17 @@
       </c>
       <c r="N20" s="11">
         <f t="shared" ref="N20:N26" si="2">(H20/(I20*J20))*M20</f>
-        <v>4.199196507262025</v>
-      </c>
-      <c r="O20" s="12">
+        <v>1.606955087974574</v>
+      </c>
+      <c r="O20" s="11">
+        <v>1.6</v>
+      </c>
+      <c r="P20" s="12">
         <f>100*((Table134[[#This Row],[themal conductivity]]/1.6)-1)</f>
-        <v>162.44978170387654</v>
-      </c>
-    </row>
-    <row r="21" spans="1:16" x14ac:dyDescent="0.3">
+        <v>0.43469299841085718</v>
+      </c>
+    </row>
+    <row r="21" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>31</v>
       </c>
@@ -1477,7 +1635,7 @@
         <v>12.566370614359172</v>
       </c>
       <c r="J21" s="14">
-        <v>0.99</v>
+        <v>2.58</v>
       </c>
       <c r="K21" s="3">
         <v>600</v>
@@ -1491,14 +1649,17 @@
       </c>
       <c r="N21" s="11">
         <f t="shared" si="2"/>
-        <v>4.1984542250511456</v>
-      </c>
-      <c r="O21" s="12">
+        <v>1.6110347607754398</v>
+      </c>
+      <c r="O21" s="11">
+        <v>1.6</v>
+      </c>
+      <c r="P21" s="12">
         <f>100*((Table134[[#This Row],[themal conductivity]]/1.6)-1)</f>
-        <v>162.40338906569659</v>
-      </c>
-    </row>
-    <row r="22" spans="1:16" x14ac:dyDescent="0.3">
+        <v>0.68967254846499237</v>
+      </c>
+    </row>
+    <row r="22" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>32</v>
       </c>
@@ -1531,7 +1692,7 @@
         <v>12.566370614359172</v>
       </c>
       <c r="J22" s="14">
-        <v>0.67</v>
+        <v>1.75</v>
       </c>
       <c r="K22" s="3">
         <v>600</v>
@@ -1545,14 +1706,17 @@
       </c>
       <c r="N22" s="11">
         <f t="shared" si="2"/>
-        <v>4.2073442019776088</v>
-      </c>
-      <c r="O22" s="12">
+        <v>1.6108117801857129</v>
+      </c>
+      <c r="O22" s="11">
+        <v>1.6</v>
+      </c>
+      <c r="P22" s="12">
         <f>100*((Table134[[#This Row],[themal conductivity]]/1.6)-1)</f>
-        <v>162.95901262360056</v>
-      </c>
-    </row>
-    <row r="23" spans="1:16" x14ac:dyDescent="0.3">
+        <v>0.67573626160704059</v>
+      </c>
+    </row>
+    <row r="23" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>33</v>
       </c>
@@ -1585,7 +1749,7 @@
         <v>12.566370614359172</v>
       </c>
       <c r="J23" s="14">
-        <v>0.41</v>
+        <v>1.08</v>
       </c>
       <c r="K23" s="3">
         <v>600</v>
@@ -1599,14 +1763,17 @@
       </c>
       <c r="N23" s="11">
         <f t="shared" si="2"/>
-        <v>4.2445171037123544</v>
-      </c>
-      <c r="O23" s="12">
+        <v>1.6113444560389489</v>
+      </c>
+      <c r="O23" s="11">
+        <v>1.6</v>
+      </c>
+      <c r="P23" s="12">
         <f>100*((Table134[[#This Row],[themal conductivity]]/1.6)-1)</f>
-        <v>165.28231898202216</v>
-      </c>
-    </row>
-    <row r="24" spans="1:16" x14ac:dyDescent="0.3">
+        <v>0.70902850243430571</v>
+      </c>
+    </row>
+    <row r="24" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>34</v>
       </c>
@@ -1639,7 +1806,7 @@
         <v>12.566370614359172</v>
       </c>
       <c r="J24" s="14">
-        <v>0.22</v>
+        <v>0.56999999999999995</v>
       </c>
       <c r="K24" s="3">
         <v>600</v>
@@ -1653,14 +1820,17 @@
       </c>
       <c r="N24" s="11">
         <f t="shared" si="2"/>
-        <v>4.1839267017810737</v>
-      </c>
-      <c r="O24" s="12">
+        <v>1.614848902441818</v>
+      </c>
+      <c r="O24" s="11">
+        <v>1.6</v>
+      </c>
+      <c r="P24" s="12">
         <f>100*((Table134[[#This Row],[themal conductivity]]/1.6)-1)</f>
-        <v>161.49541886131709</v>
-      </c>
-    </row>
-    <row r="25" spans="1:16" x14ac:dyDescent="0.3">
+        <v>0.92805640261361955</v>
+      </c>
+    </row>
+    <row r="25" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>35</v>
       </c>
@@ -1693,7 +1863,7 @@
         <v>12.566370614359172</v>
       </c>
       <c r="J25" s="14">
-        <v>0.09</v>
+        <v>0.22</v>
       </c>
       <c r="K25" s="3">
         <v>600</v>
@@ -1707,14 +1877,17 @@
       </c>
       <c r="N25" s="11">
         <f t="shared" si="2"/>
-        <v>3.9950688992701218</v>
-      </c>
-      <c r="O25" s="12">
+        <v>1.634346367883232</v>
+      </c>
+      <c r="O25" s="11">
+        <v>1.6</v>
+      </c>
+      <c r="P25" s="12">
         <f>100*((Table134[[#This Row],[themal conductivity]]/1.6)-1)</f>
-        <v>149.6918062043826</v>
-      </c>
-    </row>
-    <row r="26" spans="1:16" x14ac:dyDescent="0.3">
+        <v>2.1466479927019888</v>
+      </c>
+    </row>
+    <row r="26" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>36</v>
       </c>
@@ -1747,7 +1920,7 @@
         <v>12.566370614359172</v>
       </c>
       <c r="J26" s="14">
-        <v>0.01</v>
+        <v>0.04</v>
       </c>
       <c r="K26" s="3">
         <v>600</v>
@@ -1761,14 +1934,797 @@
       </c>
       <c r="N26" s="11">
         <f t="shared" si="2"/>
-        <v>5.7528992149489753</v>
-      </c>
-      <c r="O26" s="12">
+        <v>1.4382248037372438</v>
+      </c>
+      <c r="O26" s="11">
+        <v>1.6</v>
+      </c>
+      <c r="P26" s="12">
         <f>100*((Table134[[#This Row],[themal conductivity]]/1.6)-1)</f>
-        <v>259.55620093431094</v>
+        <v>-10.110949766422262</v>
+      </c>
+    </row>
+    <row r="27" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="B27" s="3"/>
+      <c r="C27" s="3"/>
+      <c r="D27" s="5"/>
+      <c r="E27" s="5"/>
+      <c r="F27" s="13"/>
+      <c r="G27" s="9"/>
+      <c r="H27" s="13"/>
+      <c r="I27" s="13"/>
+      <c r="J27" s="13"/>
+      <c r="K27" s="3"/>
+      <c r="L27" s="3"/>
+      <c r="M27" s="13"/>
+      <c r="N27" s="5"/>
+      <c r="O27" s="11"/>
+      <c r="P27" s="15"/>
+    </row>
+    <row r="28" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A28" s="2"/>
+      <c r="B28" s="6"/>
+      <c r="C28" s="6"/>
+      <c r="D28" s="6"/>
+      <c r="E28" s="6"/>
+      <c r="F28" s="7"/>
+      <c r="G28" s="7"/>
+      <c r="H28" s="7"/>
+      <c r="I28" s="7"/>
+      <c r="J28" s="7"/>
+      <c r="K28" s="6"/>
+      <c r="L28" s="6"/>
+      <c r="M28" s="7"/>
+      <c r="N28" s="6"/>
+      <c r="O28" s="6"/>
+      <c r="P28" s="2"/>
+    </row>
+    <row r="29" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A29" s="1"/>
+      <c r="B29" s="3"/>
+      <c r="C29" s="3"/>
+      <c r="D29" s="3"/>
+      <c r="E29" s="5"/>
+      <c r="F29" s="3"/>
+      <c r="G29" s="3"/>
+      <c r="H29" s="3"/>
+      <c r="I29" s="4"/>
+      <c r="J29" s="3"/>
+      <c r="K29" s="3"/>
+      <c r="L29" s="3"/>
+      <c r="M29" s="4"/>
+      <c r="N29" s="5"/>
+      <c r="O29" s="5"/>
+    </row>
+    <row r="30" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A30" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="B30" s="17" t="s">
+        <v>27</v>
+      </c>
+      <c r="C30" s="17" t="s">
+        <v>51</v>
+      </c>
+      <c r="D30" s="17" t="s">
+        <v>43</v>
+      </c>
+      <c r="E30" s="17" t="s">
+        <v>58</v>
+      </c>
+      <c r="F30" s="17" t="s">
+        <v>48</v>
+      </c>
+      <c r="G30" s="17" t="s">
+        <v>56</v>
+      </c>
+      <c r="H30" s="17" t="s">
+        <v>53</v>
+      </c>
+      <c r="I30" s="17" t="s">
+        <v>37</v>
+      </c>
+      <c r="J30" s="17" t="s">
+        <v>28</v>
+      </c>
+      <c r="K30" s="17" t="s">
+        <v>38</v>
+      </c>
+      <c r="L30" s="17" t="s">
+        <v>39</v>
+      </c>
+      <c r="M30" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="N30" s="17" t="s">
+        <v>41</v>
+      </c>
+      <c r="O30" s="17" t="s">
+        <v>60</v>
+      </c>
+      <c r="P30" s="18" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="31" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A31" s="19" t="s">
+        <v>3</v>
+      </c>
+      <c r="B31" s="20" t="s">
+        <v>44</v>
+      </c>
+      <c r="C31" s="20" t="s">
+        <v>50</v>
+      </c>
+      <c r="D31" s="20" t="s">
+        <v>45</v>
+      </c>
+      <c r="E31" s="21" t="s">
+        <v>52</v>
+      </c>
+      <c r="F31" s="20" t="s">
+        <v>49</v>
+      </c>
+      <c r="G31" s="20" t="s">
+        <v>3</v>
+      </c>
+      <c r="H31" s="20" t="s">
+        <v>49</v>
+      </c>
+      <c r="I31" s="22" t="s">
+        <v>46</v>
+      </c>
+      <c r="J31" s="20" t="s">
+        <v>47</v>
+      </c>
+      <c r="K31" s="20" t="s">
+        <v>57</v>
+      </c>
+      <c r="L31" s="20" t="s">
+        <v>57</v>
+      </c>
+      <c r="M31" s="22" t="s">
+        <v>3</v>
+      </c>
+      <c r="N31" s="21" t="s">
+        <v>7</v>
+      </c>
+      <c r="O31" s="21" t="s">
+        <v>7</v>
+      </c>
+      <c r="P31" s="23" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="32" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A32" s="23" t="s">
+        <v>59</v>
+      </c>
+      <c r="B32" s="20">
+        <v>230</v>
+      </c>
+      <c r="C32" s="20">
+        <v>1.47</v>
+      </c>
+      <c r="D32" s="21">
+        <v>28</v>
+      </c>
+      <c r="E32" s="21">
+        <f>C32*D32</f>
+        <v>41.16</v>
+      </c>
+      <c r="F32" s="24">
+        <f>B32^2/(E32*D32)</f>
+        <v>45.901013466611133</v>
+      </c>
+      <c r="G32" s="25">
+        <v>2</v>
+      </c>
+      <c r="H32" s="24">
+        <f>F32*G32</f>
+        <v>91.802026933222265</v>
+      </c>
+      <c r="I32" s="24">
+        <f>4*PI()</f>
+        <v>12.566370614359172</v>
+      </c>
+      <c r="J32" s="26">
+        <v>7.39</v>
+      </c>
+      <c r="K32" s="20">
+        <v>600</v>
+      </c>
+      <c r="L32" s="20">
+        <v>1700</v>
+      </c>
+      <c r="M32" s="27">
+        <f>LN(L32/K32)</f>
+        <v>1.0414538748281612</v>
+      </c>
+      <c r="N32" s="28">
+        <f>(H32/(I32*J32))*M32</f>
+        <v>1.029527633527743</v>
+      </c>
+      <c r="O32" s="28">
+        <v>1</v>
+      </c>
+      <c r="P32" s="29">
+        <f>100*((N32/O32)-1)</f>
+        <v>2.9527633527743014</v>
+      </c>
+    </row>
+    <row r="33" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A33" s="23" t="s">
+        <v>61</v>
+      </c>
+      <c r="B33" s="20">
+        <v>230</v>
+      </c>
+      <c r="C33" s="20">
+        <v>1.47</v>
+      </c>
+      <c r="D33" s="21">
+        <v>28</v>
+      </c>
+      <c r="E33" s="21">
+        <f t="shared" ref="E33:E42" si="3">C33*D33</f>
+        <v>41.16</v>
+      </c>
+      <c r="F33" s="24">
+        <f t="shared" ref="F33:F42" si="4">B33^2/(E33*D33)</f>
+        <v>45.901013466611133</v>
+      </c>
+      <c r="G33" s="25">
+        <v>2</v>
+      </c>
+      <c r="H33" s="24">
+        <f t="shared" ref="H33:H42" si="5">F33*G33</f>
+        <v>91.802026933222265</v>
+      </c>
+      <c r="I33" s="24">
+        <f t="shared" ref="I33:I42" si="6">4*PI()</f>
+        <v>12.566370614359172</v>
+      </c>
+      <c r="J33" s="26">
+        <v>6.22</v>
+      </c>
+      <c r="K33" s="20">
+        <v>600</v>
+      </c>
+      <c r="L33" s="20">
+        <v>1700</v>
+      </c>
+      <c r="M33" s="27">
+        <f t="shared" ref="M33:M39" si="7">LN(L33/K33)</f>
+        <v>1.0414538748281612</v>
+      </c>
+      <c r="N33" s="28">
+        <f t="shared" ref="N33:N42" si="8">(H33/(I33*J33))*M33</f>
+        <v>1.2231847607347299</v>
+      </c>
+      <c r="O33" s="28">
+        <v>1.2</v>
+      </c>
+      <c r="P33" s="29">
+        <f t="shared" ref="P33:P42" si="9">100*((N33/O33)-1)</f>
+        <v>1.9320633945608234</v>
+      </c>
+    </row>
+    <row r="34" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A34" s="23" t="s">
+        <v>62</v>
+      </c>
+      <c r="B34" s="20">
+        <v>230</v>
+      </c>
+      <c r="C34" s="20">
+        <v>1.47</v>
+      </c>
+      <c r="D34" s="21">
+        <v>28</v>
+      </c>
+      <c r="E34" s="21">
+        <f t="shared" si="3"/>
+        <v>41.16</v>
+      </c>
+      <c r="F34" s="24">
+        <f t="shared" si="4"/>
+        <v>45.901013466611133</v>
+      </c>
+      <c r="G34" s="25">
+        <v>2</v>
+      </c>
+      <c r="H34" s="24">
+        <f t="shared" si="5"/>
+        <v>91.802026933222265</v>
+      </c>
+      <c r="I34" s="24">
+        <f t="shared" si="6"/>
+        <v>12.566370614359172</v>
+      </c>
+      <c r="J34" s="26">
+        <v>5.37</v>
+      </c>
+      <c r="K34" s="20">
+        <v>600</v>
+      </c>
+      <c r="L34" s="20">
+        <v>1700</v>
+      </c>
+      <c r="M34" s="27">
+        <f t="shared" si="7"/>
+        <v>1.0414538748281612</v>
+      </c>
+      <c r="N34" s="28">
+        <f t="shared" si="8"/>
+        <v>1.4167987358975831</v>
+      </c>
+      <c r="O34" s="28">
+        <v>1.4</v>
+      </c>
+      <c r="P34" s="29">
+        <f t="shared" si="9"/>
+        <v>1.1999097069702369</v>
+      </c>
+    </row>
+    <row r="35" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A35" s="23" t="s">
+        <v>63</v>
+      </c>
+      <c r="B35" s="20">
+        <v>230</v>
+      </c>
+      <c r="C35" s="20">
+        <v>1.47</v>
+      </c>
+      <c r="D35" s="21">
+        <v>28</v>
+      </c>
+      <c r="E35" s="21">
+        <f t="shared" si="3"/>
+        <v>41.16</v>
+      </c>
+      <c r="F35" s="24">
+        <f t="shared" si="4"/>
+        <v>45.901013466611133</v>
+      </c>
+      <c r="G35" s="25">
+        <v>2</v>
+      </c>
+      <c r="H35" s="24">
+        <f t="shared" si="5"/>
+        <v>91.802026933222265</v>
+      </c>
+      <c r="I35" s="24">
+        <f t="shared" si="6"/>
+        <v>12.566370614359172</v>
+      </c>
+      <c r="J35" s="26">
+        <v>4.7300000000000004</v>
+      </c>
+      <c r="K35" s="20">
+        <v>600</v>
+      </c>
+      <c r="L35" s="20">
+        <v>1700</v>
+      </c>
+      <c r="M35" s="27">
+        <f t="shared" si="7"/>
+        <v>1.0414538748281612</v>
+      </c>
+      <c r="N35" s="28">
+        <f t="shared" si="8"/>
+        <v>1.6085008904376361</v>
+      </c>
+      <c r="O35" s="28">
+        <v>1.6</v>
+      </c>
+      <c r="P35" s="29">
+        <f t="shared" si="9"/>
+        <v>0.53130565235224303</v>
+      </c>
+    </row>
+    <row r="36" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A36" s="23" t="s">
+        <v>64</v>
+      </c>
+      <c r="B36" s="20">
+        <v>230</v>
+      </c>
+      <c r="C36" s="20">
+        <v>1.47</v>
+      </c>
+      <c r="D36" s="21">
+        <v>28</v>
+      </c>
+      <c r="E36" s="21">
+        <f t="shared" si="3"/>
+        <v>41.16</v>
+      </c>
+      <c r="F36" s="24">
+        <f t="shared" si="4"/>
+        <v>45.901013466611133</v>
+      </c>
+      <c r="G36" s="25">
+        <v>2</v>
+      </c>
+      <c r="H36" s="24">
+        <f t="shared" si="5"/>
+        <v>91.802026933222265</v>
+      </c>
+      <c r="I36" s="24">
+        <f t="shared" si="6"/>
+        <v>12.566370614359172</v>
+      </c>
+      <c r="J36" s="26">
+        <v>4.22</v>
+      </c>
+      <c r="K36" s="20">
+        <v>600</v>
+      </c>
+      <c r="L36" s="20">
+        <v>1700</v>
+      </c>
+      <c r="M36" s="27">
+        <f t="shared" si="7"/>
+        <v>1.0414538748281612</v>
+      </c>
+      <c r="N36" s="28">
+        <f t="shared" si="8"/>
+        <v>1.8028931781445545</v>
+      </c>
+      <c r="O36" s="28">
+        <v>1.8</v>
+      </c>
+      <c r="P36" s="29">
+        <f t="shared" si="9"/>
+        <v>0.16073211914191532</v>
+      </c>
+    </row>
+    <row r="37" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A37" s="23" t="s">
+        <v>65</v>
+      </c>
+      <c r="B37" s="20">
+        <v>230</v>
+      </c>
+      <c r="C37" s="20">
+        <v>1.47</v>
+      </c>
+      <c r="D37" s="21">
+        <v>28</v>
+      </c>
+      <c r="E37" s="21">
+        <f t="shared" si="3"/>
+        <v>41.16</v>
+      </c>
+      <c r="F37" s="24">
+        <f t="shared" si="4"/>
+        <v>45.901013466611133</v>
+      </c>
+      <c r="G37" s="25">
+        <v>2</v>
+      </c>
+      <c r="H37" s="24">
+        <f t="shared" si="5"/>
+        <v>91.802026933222265</v>
+      </c>
+      <c r="I37" s="24">
+        <f t="shared" si="6"/>
+        <v>12.566370614359172</v>
+      </c>
+      <c r="J37" s="26">
+        <v>3.81</v>
+      </c>
+      <c r="K37" s="20">
+        <v>600</v>
+      </c>
+      <c r="L37" s="20">
+        <v>1700</v>
+      </c>
+      <c r="M37" s="27">
+        <f t="shared" si="7"/>
+        <v>1.0414538748281612</v>
+      </c>
+      <c r="N37" s="28">
+        <f t="shared" si="8"/>
+        <v>1.9969053049265144</v>
+      </c>
+      <c r="O37" s="28">
+        <v>2</v>
+      </c>
+      <c r="P37" s="29">
+        <f t="shared" si="9"/>
+        <v>-0.15473475367427936</v>
+      </c>
+    </row>
+    <row r="38" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A38" s="23" t="s">
+        <v>66</v>
+      </c>
+      <c r="B38" s="20">
+        <v>230</v>
+      </c>
+      <c r="C38" s="20">
+        <v>1.47</v>
+      </c>
+      <c r="D38" s="21">
+        <v>28</v>
+      </c>
+      <c r="E38" s="21">
+        <f t="shared" si="3"/>
+        <v>41.16</v>
+      </c>
+      <c r="F38" s="24">
+        <f t="shared" si="4"/>
+        <v>45.901013466611133</v>
+      </c>
+      <c r="G38" s="25">
+        <v>2</v>
+      </c>
+      <c r="H38" s="24">
+        <f t="shared" si="5"/>
+        <v>91.802026933222265</v>
+      </c>
+      <c r="I38" s="24">
+        <f t="shared" si="6"/>
+        <v>12.566370614359172</v>
+      </c>
+      <c r="J38" s="26">
+        <v>3.48</v>
+      </c>
+      <c r="K38" s="20">
+        <v>600</v>
+      </c>
+      <c r="L38" s="20">
+        <v>1700</v>
+      </c>
+      <c r="M38" s="27">
+        <f t="shared" si="7"/>
+        <v>1.0414538748281612</v>
+      </c>
+      <c r="N38" s="28">
+        <f t="shared" si="8"/>
+        <v>2.1862670148764427</v>
+      </c>
+      <c r="O38" s="28">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="P38" s="29">
+        <f t="shared" si="9"/>
+        <v>-0.62422659652533463</v>
+      </c>
+    </row>
+    <row r="39" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A39" s="23" t="s">
+        <v>67</v>
+      </c>
+      <c r="B39" s="20">
+        <v>230</v>
+      </c>
+      <c r="C39" s="20">
+        <v>1.47</v>
+      </c>
+      <c r="D39" s="21">
+        <v>28</v>
+      </c>
+      <c r="E39" s="21">
+        <f t="shared" si="3"/>
+        <v>41.16</v>
+      </c>
+      <c r="F39" s="24">
+        <f t="shared" si="4"/>
+        <v>45.901013466611133</v>
+      </c>
+      <c r="G39" s="25">
+        <v>2</v>
+      </c>
+      <c r="H39" s="24">
+        <f t="shared" si="5"/>
+        <v>91.802026933222265</v>
+      </c>
+      <c r="I39" s="24">
+        <f t="shared" si="6"/>
+        <v>12.566370614359172</v>
+      </c>
+      <c r="J39" s="26">
+        <v>3.2</v>
+      </c>
+      <c r="K39" s="20">
+        <v>600</v>
+      </c>
+      <c r="L39" s="20">
+        <v>1700</v>
+      </c>
+      <c r="M39" s="27">
+        <f t="shared" si="7"/>
+        <v>1.0414538748281612</v>
+      </c>
+      <c r="N39" s="28">
+        <f t="shared" si="8"/>
+        <v>2.3775653786781317</v>
+      </c>
+      <c r="O39" s="28">
+        <v>2.4</v>
+      </c>
+      <c r="P39" s="29">
+        <f t="shared" si="9"/>
+        <v>-0.93477588841117676</v>
+      </c>
+    </row>
+    <row r="40" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A40" s="23" t="s">
+        <v>68</v>
+      </c>
+      <c r="B40" s="20">
+        <v>230</v>
+      </c>
+      <c r="C40" s="20">
+        <v>1.47</v>
+      </c>
+      <c r="D40" s="21">
+        <v>28</v>
+      </c>
+      <c r="E40" s="21">
+        <f t="shared" si="3"/>
+        <v>41.16</v>
+      </c>
+      <c r="F40" s="24">
+        <f t="shared" si="4"/>
+        <v>45.901013466611133</v>
+      </c>
+      <c r="G40" s="25">
+        <v>2</v>
+      </c>
+      <c r="H40" s="24">
+        <f t="shared" si="5"/>
+        <v>91.802026933222265</v>
+      </c>
+      <c r="I40" s="24">
+        <f t="shared" si="6"/>
+        <v>12.566370614359172</v>
+      </c>
+      <c r="J40" s="30">
+        <v>2.96</v>
+      </c>
+      <c r="K40" s="20">
+        <v>600</v>
+      </c>
+      <c r="L40" s="20">
+        <v>1700</v>
+      </c>
+      <c r="M40" s="27">
+        <f t="shared" ref="M40:M42" si="10">LN(L40/K40)</f>
+        <v>1.0414538748281612</v>
+      </c>
+      <c r="N40" s="28">
+        <f t="shared" si="8"/>
+        <v>2.5703409499223042</v>
+      </c>
+      <c r="O40" s="31">
+        <v>2.6</v>
+      </c>
+      <c r="P40" s="29">
+        <f t="shared" si="9"/>
+        <v>-1.1407326952959984</v>
+      </c>
+    </row>
+    <row r="41" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A41" s="23" t="s">
+        <v>69</v>
+      </c>
+      <c r="B41" s="20">
+        <v>230</v>
+      </c>
+      <c r="C41" s="20">
+        <v>1.47</v>
+      </c>
+      <c r="D41" s="21">
+        <v>28</v>
+      </c>
+      <c r="E41" s="21">
+        <f t="shared" si="3"/>
+        <v>41.16</v>
+      </c>
+      <c r="F41" s="24">
+        <f t="shared" si="4"/>
+        <v>45.901013466611133</v>
+      </c>
+      <c r="G41" s="25">
+        <v>2</v>
+      </c>
+      <c r="H41" s="24">
+        <f t="shared" si="5"/>
+        <v>91.802026933222265</v>
+      </c>
+      <c r="I41" s="24">
+        <f t="shared" si="6"/>
+        <v>12.566370614359172</v>
+      </c>
+      <c r="J41" s="30">
+        <v>2.75</v>
+      </c>
+      <c r="K41" s="20">
+        <v>600</v>
+      </c>
+      <c r="L41" s="20">
+        <v>1700</v>
+      </c>
+      <c r="M41" s="27">
+        <f t="shared" si="10"/>
+        <v>1.0414538748281612</v>
+      </c>
+      <c r="N41" s="28">
+        <f t="shared" si="8"/>
+        <v>2.7666215315527349</v>
+      </c>
+      <c r="O41" s="31">
+        <v>2.8</v>
+      </c>
+      <c r="P41" s="29">
+        <f t="shared" si="9"/>
+        <v>-1.192088158830884</v>
+      </c>
+    </row>
+    <row r="42" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A42" s="23" t="s">
+        <v>70</v>
+      </c>
+      <c r="B42" s="20">
+        <v>230</v>
+      </c>
+      <c r="C42" s="20">
+        <v>1.47</v>
+      </c>
+      <c r="D42" s="21">
+        <v>28</v>
+      </c>
+      <c r="E42" s="21">
+        <f t="shared" si="3"/>
+        <v>41.16</v>
+      </c>
+      <c r="F42" s="24">
+        <f t="shared" si="4"/>
+        <v>45.901013466611133</v>
+      </c>
+      <c r="G42" s="25">
+        <v>2</v>
+      </c>
+      <c r="H42" s="24">
+        <f t="shared" si="5"/>
+        <v>91.802026933222265</v>
+      </c>
+      <c r="I42" s="24">
+        <f t="shared" si="6"/>
+        <v>12.566370614359172</v>
+      </c>
+      <c r="J42" s="30">
+        <v>2.58</v>
+      </c>
+      <c r="K42" s="20">
+        <v>600</v>
+      </c>
+      <c r="L42" s="20">
+        <v>1700</v>
+      </c>
+      <c r="M42" s="27">
+        <f t="shared" si="10"/>
+        <v>1.0414538748281612</v>
+      </c>
+      <c r="N42" s="28">
+        <f t="shared" si="8"/>
+        <v>2.9489182991356668</v>
+      </c>
+      <c r="O42" s="31">
+        <v>3</v>
+      </c>
+      <c r="P42" s="29">
+        <f t="shared" si="9"/>
+        <v>-1.7027233621444426</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="7" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" r:id="rId1"/>
   <drawing r:id="rId2"/>

</xml_diff>